<commit_message>
Terminal run evening 2026-10-02-1439
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Emergency_and_Rescue.xlsx
+++ b/results/auto_Cape_Town_Emergency_and_Rescue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="30">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>info@firevolunteers.co.za</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -471,6 +474,9 @@
       <c r="D2" t="s">
         <v>19</v>
       </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -485,6 +491,9 @@
       <c r="D3" t="s">
         <v>20</v>
       </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -499,6 +508,9 @@
       <c r="D4" t="s">
         <v>21</v>
       </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -513,6 +525,9 @@
       <c r="D5" t="s">
         <v>22</v>
       </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -527,6 +542,9 @@
       <c r="D6" t="s">
         <v>23</v>
       </c>
+      <c r="G6" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -541,6 +559,9 @@
       <c r="D7" t="s">
         <v>24</v>
       </c>
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -555,6 +576,9 @@
       <c r="D8" t="s">
         <v>25</v>
       </c>
+      <c r="G8" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -569,6 +593,9 @@
       <c r="D9" t="s">
         <v>26</v>
       </c>
+      <c r="G9" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -583,6 +610,9 @@
       <c r="D10" t="s">
         <v>27</v>
       </c>
+      <c r="G10" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -596,6 +626,9 @@
       </c>
       <c r="D11" t="s">
         <v>28</v>
+      </c>
+      <c r="G11" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>